<commit_message>
#56 HUB Design BOM Updated File.
</commit_message>
<xml_diff>
--- a/Deliverables/HUB/BOM/eSpark_Ezlo_Voice_AssistantHUB.xlsx
+++ b/Deliverables/HUB/BOM/eSpark_Ezlo_Voice_AssistantHUB.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverables\HUB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D7FC4A-B2CB-465D-8621-63C357B62A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B94B6F8D-71B9-455E-B07E-5018962636D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1862,9 +1862,6 @@
     <t>C386736</t>
   </si>
   <si>
-    <t>C3, C61, C142, C144, C241, C245, C29</t>
-  </si>
-  <si>
     <t>RK808 QFN68 K808 Power management chip</t>
   </si>
   <si>
@@ -1874,12 +1871,6 @@
     <t>C23, C25, C35, C36, C37, C38, C39, C40, C41, C42, C47, C57, C58, C60, C67, C78, C82, C96, C105, C124, C161, C162, C163, C174, C179, C182, C230</t>
   </si>
   <si>
-    <t>R1, R9, R12, R13, R19, R21, R24, R27, R32, R39, R40, R42, R44, R48, R56, R66, R96, R97, R98, R99, R101, R102, R104, R106, R107, R109, R110, R111, R113, R118, R123, R124, R125, R15, R58, R59, R117</t>
-  </si>
-  <si>
-    <t>R2, R10, R11, R116, R120, R121, R122, R30, R31, R37</t>
-  </si>
-  <si>
     <t>Need Custom Supplier Quotation</t>
   </si>
   <si>
@@ -1905,6 +1896,15 @@
   </si>
   <si>
     <t>C307331</t>
+  </si>
+  <si>
+    <t>C3, C29, C61, C142, C144, C241, C245</t>
+  </si>
+  <si>
+    <t>R1, R9, R12, R13, R15, R19, R21, R24, R27, R32, R39, R40, R42, R44, R48, R56, R58, R59, R66, R96, R97, R98, R99, R101, R102, R104, R106, R107, R109, R110, R111, R113, R117, R118, R123, R124, R125</t>
+  </si>
+  <si>
+    <t>R2, R10, R11, R30, R31, R37, R116, R120, R121, R122</t>
   </si>
 </sst>
 </file>
@@ -2610,6 +2610,15 @@
     <xf numFmtId="166" fontId="15" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2641,15 +2650,6 @@
     <xf numFmtId="0" fontId="24" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3001,8 +3001,8 @@
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="30.85546875" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -3027,15 +3027,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="79"/>
-      <c r="R1" s="79"/>
-      <c r="S1" s="80"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="83"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="56" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="57" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -3085,7 +3085,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="81"/>
+      <c r="S3" s="84"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="58" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -3110,7 +3110,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="82"/>
+      <c r="S4" s="85"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3135,7 +3135,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="82"/>
+      <c r="S5" s="85"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -3156,7 +3156,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="82"/>
+      <c r="S6" s="85"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -3177,7 +3177,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="82"/>
+      <c r="S7" s="85"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -3198,7 +3198,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="82"/>
+      <c r="S8" s="85"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3491,7 +3491,7 @@
         <v>467</v>
       </c>
       <c r="D14" s="46" t="s">
-        <v>610</v>
+        <v>622</v>
       </c>
       <c r="E14" s="47" t="s">
         <v>116</v>
@@ -3715,7 +3715,7 @@
         <v>467</v>
       </c>
       <c r="D18" s="46" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="E18" s="47" t="s">
         <v>120</v>
@@ -4110,22 +4110,22 @@
         <v>581</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="F25" s="50" t="s">
         <v>224</v>
       </c>
       <c r="G25" s="65" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="H25" s="50" t="s">
         <v>354</v>
       </c>
       <c r="I25" s="50" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="J25" s="50" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="K25" s="50" t="s">
         <v>406</v>
@@ -6518,7 +6518,7 @@
         <v>475</v>
       </c>
       <c r="D68" s="46" t="s">
-        <v>614</v>
+        <v>623</v>
       </c>
       <c r="E68" s="47" t="s">
         <v>169</v>
@@ -6918,7 +6918,7 @@
       <c r="F75" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="G75" s="91" t="s">
+      <c r="G75" s="81" t="s">
         <v>315</v>
       </c>
       <c r="H75" s="50" t="s">
@@ -7358,7 +7358,7 @@
         <v>475</v>
       </c>
       <c r="D83" s="50" t="s">
-        <v>615</v>
+        <v>624</v>
       </c>
       <c r="E83" s="51" t="s">
         <v>184</v>
@@ -7702,7 +7702,7 @@
       <c r="F89" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="G89" s="91" t="s">
+      <c r="G89" s="81" t="s">
         <v>329</v>
       </c>
       <c r="H89" s="50" t="s">
@@ -8754,7 +8754,7 @@
         <v>99</v>
       </c>
       <c r="E108" s="73" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F108" s="72" t="s">
         <v>264</v>
@@ -8784,8 +8784,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R108" s="90" t="s">
-        <v>616</v>
+      <c r="R108" s="80" t="s">
+        <v>613</v>
       </c>
       <c r="S108" s="76"/>
     </row>
@@ -8802,7 +8802,7 @@
         <v>100</v>
       </c>
       <c r="E109" s="68" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F109" s="67" t="s">
         <v>607</v>
@@ -8832,10 +8832,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R109" s="90" t="s">
-        <v>616</v>
-      </c>
-      <c r="S109" s="89"/>
+      <c r="R109" s="80" t="s">
+        <v>613</v>
+      </c>
+      <c r="S109" s="79"/>
     </row>
     <row r="110" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1"/>
@@ -9160,10 +9160,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R115" s="90" t="s">
-        <v>616</v>
-      </c>
-      <c r="S115" s="89"/>
+      <c r="R115" s="80" t="s">
+        <v>613</v>
+      </c>
+      <c r="S115" s="79"/>
     </row>
     <row r="116" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1"/>
@@ -9403,17 +9403,17 @@
       <c r="K120" s="37"/>
       <c r="L120" s="37"/>
       <c r="M120" s="37"/>
-      <c r="N120" s="87" t="s">
-        <v>619</v>
-      </c>
-      <c r="O120" s="88"/>
-      <c r="P120" s="88"/>
+      <c r="N120" s="90" t="s">
+        <v>616</v>
+      </c>
+      <c r="O120" s="91"/>
+      <c r="P120" s="91"/>
       <c r="Q120" s="77">
         <f>SUM(Q10:Q119)</f>
         <v>568.75290000000007</v>
       </c>
-      <c r="R120" s="83"/>
-      <c r="S120" s="84"/>
+      <c r="R120" s="86"/>
+      <c r="S120" s="87"/>
     </row>
     <row r="121" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1"/>
@@ -9429,17 +9429,17 @@
       <c r="K121" s="10"/>
       <c r="L121" s="10"/>
       <c r="M121" s="10"/>
-      <c r="N121" s="87" t="s">
-        <v>620</v>
-      </c>
-      <c r="O121" s="88"/>
-      <c r="P121" s="88"/>
+      <c r="N121" s="90" t="s">
+        <v>617</v>
+      </c>
+      <c r="O121" s="91"/>
+      <c r="P121" s="91"/>
       <c r="Q121" s="78">
         <f>Q120/10</f>
         <v>56.875290000000007</v>
       </c>
-      <c r="R121" s="85"/>
-      <c r="S121" s="86"/>
+      <c r="R121" s="88"/>
+      <c r="S121" s="89"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
#56 Updated BOM files.
</commit_message>
<xml_diff>
--- a/Deliverables/HUB/BOM/eSpark_Ezlo_Voice_AssistantHUB.xlsx
+++ b/Deliverables/HUB/BOM/eSpark_Ezlo_Voice_AssistantHUB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverables\HUB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B94B6F8D-71B9-455E-B07E-5018962636D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C54531-BCBC-45B0-A66C-C2CA7F929DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="626">
   <si>
     <t>Component list</t>
   </si>
@@ -1871,9 +1871,6 @@
     <t>C23, C25, C35, C36, C37, C38, C39, C40, C41, C42, C47, C57, C58, C60, C67, C78, C82, C96, C105, C124, C161, C162, C163, C174, C179, C182, C230</t>
   </si>
   <si>
-    <t>Need Custom Supplier Quotation</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [HUB_Design]</t>
   </si>
   <si>
@@ -1905,6 +1902,12 @@
   </si>
   <si>
     <t>R2, R10, R11, R30, R31, R37, R116, R120, R121, R122</t>
+  </si>
+  <si>
+    <t>Karen Quote</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
   </si>
 </sst>
 </file>
@@ -2392,7 +2395,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2595,9 +2598,6 @@
     <xf numFmtId="0" fontId="18" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="18" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2650,6 +2650,15 @@
     <xf numFmtId="0" fontId="24" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3009,7 +3018,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -3027,15 +3036,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="82"/>
-      <c r="R1" s="82"/>
-      <c r="S1" s="83"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="82"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3046,7 +3055,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="56" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -3071,7 +3080,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="57" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -3085,7 +3094,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="84"/>
+      <c r="S3" s="83"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3096,7 +3105,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="58" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -3110,7 +3119,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="85"/>
+      <c r="S4" s="84"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3135,7 +3144,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="85"/>
+      <c r="S5" s="84"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -3156,7 +3165,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="85"/>
+      <c r="S6" s="84"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -3177,7 +3186,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="85"/>
+      <c r="S7" s="84"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -3198,7 +3207,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="85"/>
+      <c r="S8" s="84"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3491,7 +3500,7 @@
         <v>467</v>
       </c>
       <c r="D14" s="46" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E14" s="47" t="s">
         <v>116</v>
@@ -4110,22 +4119,22 @@
         <v>581</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F25" s="50" t="s">
         <v>224</v>
       </c>
       <c r="G25" s="65" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="H25" s="50" t="s">
         <v>354</v>
       </c>
       <c r="I25" s="50" t="s">
+        <v>619</v>
+      </c>
+      <c r="J25" s="50" t="s">
         <v>620</v>
-      </c>
-      <c r="J25" s="50" t="s">
-        <v>621</v>
       </c>
       <c r="K25" s="50" t="s">
         <v>406</v>
@@ -6518,7 +6527,7 @@
         <v>475</v>
       </c>
       <c r="D68" s="46" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E68" s="47" t="s">
         <v>169</v>
@@ -6918,7 +6927,7 @@
       <c r="F75" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="G75" s="81" t="s">
+      <c r="G75" s="80" t="s">
         <v>315</v>
       </c>
       <c r="H75" s="50" t="s">
@@ -7358,7 +7367,7 @@
         <v>475</v>
       </c>
       <c r="D83" s="50" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E83" s="51" t="s">
         <v>184</v>
@@ -7702,7 +7711,7 @@
       <c r="F89" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="G89" s="81" t="s">
+      <c r="G89" s="80" t="s">
         <v>329</v>
       </c>
       <c r="H89" s="50" t="s">
@@ -8299,7 +8308,7 @@
       <c r="R99" s="52" t="s">
         <v>484</v>
       </c>
-      <c r="S99" s="53" t="s">
+      <c r="S99" s="92" t="s">
         <v>484</v>
       </c>
     </row>
@@ -8365,45 +8374,45 @@
         <f>ROW(B101) - ROW($B$9)</f>
         <v>92</v>
       </c>
-      <c r="C101" s="61" t="s">
+      <c r="C101" s="66" t="s">
         <v>473</v>
       </c>
-      <c r="D101" s="50" t="s">
+      <c r="D101" s="67" t="s">
         <v>92</v>
       </c>
-      <c r="E101" s="51" t="s">
+      <c r="E101" s="68" t="s">
         <v>202</v>
       </c>
-      <c r="F101" s="50" t="s">
+      <c r="F101" s="67" t="s">
         <v>580</v>
       </c>
-      <c r="G101" s="51" t="s">
+      <c r="G101" s="68" t="s">
         <v>260</v>
       </c>
-      <c r="H101" s="50" t="s">
+      <c r="H101" s="67" t="s">
         <v>388</v>
       </c>
-      <c r="I101" s="50"/>
-      <c r="J101" s="50"/>
-      <c r="K101" s="50" t="s">
-        <v>484</v>
-      </c>
-      <c r="L101" s="51">
+      <c r="I101" s="67"/>
+      <c r="J101" s="67"/>
+      <c r="K101" s="67" t="s">
+        <v>484</v>
+      </c>
+      <c r="L101" s="68">
         <v>1</v>
       </c>
-      <c r="M101" s="50">
+      <c r="M101" s="67">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N101" s="50"/>
-      <c r="O101" s="63"/>
-      <c r="P101" s="55"/>
-      <c r="Q101" s="55">
+      <c r="N101" s="67"/>
+      <c r="O101" s="69"/>
+      <c r="P101" s="70"/>
+      <c r="Q101" s="70">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="R101" s="52"/>
-      <c r="S101" s="53"/>
+      <c r="R101" s="93"/>
+      <c r="S101" s="78"/>
     </row>
     <row r="102" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1"/>
@@ -8741,7 +8750,7 @@
       <c r="R107" s="52"/>
       <c r="S107" s="53"/>
     </row>
-    <row r="108" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1"/>
       <c r="B108" s="38">
         <f t="shared" si="0"/>
@@ -8765,8 +8774,12 @@
       <c r="H108" s="72" t="s">
         <v>393</v>
       </c>
-      <c r="I108" s="72"/>
-      <c r="J108" s="72"/>
+      <c r="I108" s="72" t="s">
+        <v>484</v>
+      </c>
+      <c r="J108" s="72" t="s">
+        <v>484</v>
+      </c>
       <c r="K108" s="72" t="s">
         <v>484</v>
       </c>
@@ -8777,19 +8790,25 @@
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N108" s="72"/>
-      <c r="O108" s="74"/>
-      <c r="P108" s="75"/>
-      <c r="Q108" s="75">
+      <c r="N108" s="72">
+        <v>11</v>
+      </c>
+      <c r="O108" s="91" t="s">
+        <v>625</v>
+      </c>
+      <c r="P108" s="74">
+        <v>1.96</v>
+      </c>
+      <c r="Q108" s="74">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R108" s="80" t="s">
-        <v>613</v>
-      </c>
-      <c r="S108" s="76"/>
-    </row>
-    <row r="109" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>21.56</v>
+      </c>
+      <c r="R108" s="79" t="s">
+        <v>624</v>
+      </c>
+      <c r="S108" s="75"/>
+    </row>
+    <row r="109" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1"/>
       <c r="B109" s="38">
         <f>ROW(B109) - ROW($B$9)</f>
@@ -8813,8 +8832,12 @@
       <c r="H109" s="67" t="s">
         <v>394</v>
       </c>
-      <c r="I109" s="67"/>
-      <c r="J109" s="67"/>
+      <c r="I109" s="67" t="s">
+        <v>484</v>
+      </c>
+      <c r="J109" s="67" t="s">
+        <v>484</v>
+      </c>
       <c r="K109" s="67" t="s">
         <v>484</v>
       </c>
@@ -8825,17 +8848,23 @@
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N109" s="67"/>
-      <c r="O109" s="69"/>
-      <c r="P109" s="70"/>
+      <c r="N109" s="67">
+        <v>11</v>
+      </c>
+      <c r="O109" s="69" t="s">
+        <v>625</v>
+      </c>
+      <c r="P109" s="70">
+        <v>20.83</v>
+      </c>
       <c r="Q109" s="70">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R109" s="80" t="s">
-        <v>613</v>
-      </c>
-      <c r="S109" s="79"/>
+        <v>229.13</v>
+      </c>
+      <c r="R109" s="79" t="s">
+        <v>624</v>
+      </c>
+      <c r="S109" s="78"/>
     </row>
     <row r="110" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1"/>
@@ -9117,7 +9146,7 @@
       <c r="R114" s="48"/>
       <c r="S114" s="48"/>
     </row>
-    <row r="115" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1"/>
       <c r="B115" s="38">
         <f>ROW(B115) - ROW($B$9)</f>
@@ -9141,8 +9170,12 @@
       <c r="H115" s="67" t="s">
         <v>399</v>
       </c>
-      <c r="I115" s="67"/>
-      <c r="J115" s="67"/>
+      <c r="I115" s="67" t="s">
+        <v>484</v>
+      </c>
+      <c r="J115" s="67" t="s">
+        <v>484</v>
+      </c>
       <c r="K115" s="67" t="s">
         <v>484</v>
       </c>
@@ -9153,17 +9186,21 @@
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N115" s="67"/>
+      <c r="N115" s="67">
+        <v>11</v>
+      </c>
       <c r="O115" s="69"/>
-      <c r="P115" s="70"/>
+      <c r="P115" s="70">
+        <v>17.5</v>
+      </c>
       <c r="Q115" s="70">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R115" s="80" t="s">
-        <v>613</v>
-      </c>
-      <c r="S115" s="79"/>
+        <v>192.5</v>
+      </c>
+      <c r="R115" s="79" t="s">
+        <v>624</v>
+      </c>
+      <c r="S115" s="78"/>
     </row>
     <row r="116" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1"/>
@@ -9403,17 +9440,17 @@
       <c r="K120" s="37"/>
       <c r="L120" s="37"/>
       <c r="M120" s="37"/>
-      <c r="N120" s="90" t="s">
-        <v>616</v>
-      </c>
-      <c r="O120" s="91"/>
-      <c r="P120" s="91"/>
-      <c r="Q120" s="77">
+      <c r="N120" s="89" t="s">
+        <v>615</v>
+      </c>
+      <c r="O120" s="90"/>
+      <c r="P120" s="90"/>
+      <c r="Q120" s="76">
         <f>SUM(Q10:Q119)</f>
-        <v>568.75290000000007</v>
-      </c>
-      <c r="R120" s="86"/>
-      <c r="S120" s="87"/>
+        <v>1011.9429</v>
+      </c>
+      <c r="R120" s="85"/>
+      <c r="S120" s="86"/>
     </row>
     <row r="121" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1"/>
@@ -9429,17 +9466,17 @@
       <c r="K121" s="10"/>
       <c r="L121" s="10"/>
       <c r="M121" s="10"/>
-      <c r="N121" s="90" t="s">
-        <v>617</v>
-      </c>
-      <c r="O121" s="91"/>
-      <c r="P121" s="91"/>
-      <c r="Q121" s="78">
+      <c r="N121" s="89" t="s">
+        <v>616</v>
+      </c>
+      <c r="O121" s="90"/>
+      <c r="P121" s="90"/>
+      <c r="Q121" s="77">
         <f>Q120/10</f>
-        <v>56.875290000000007</v>
-      </c>
-      <c r="R121" s="88"/>
-      <c r="S121" s="89"/>
+        <v>101.19429</v>
+      </c>
+      <c r="R121" s="87"/>
+      <c r="S121" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>